<commit_message>
Fix homeworks 0 and 1
</commit_message>
<xml_diff>
--- a/data/processed/hw01/table_summary.xlsx
+++ b/data/processed/hw01/table_summary.xlsx
@@ -413,70 +413,85 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>pressure_mpa</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>radius_m</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>thickness_m</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>porosity_fraction</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>9.42</v>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>5</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>2</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>12</v>
       </c>
-      <c r="B3" t="n">
+      <c r="C3" t="n">
         <v>500</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>7</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>0.24</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>10.75</v>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
         <v>150.7142857142857</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>4.5</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>0.195</v>
       </c>
     </row>

</xml_diff>